<commit_message>
Update dashboards and data template
</commit_message>
<xml_diff>
--- a/Data template.xlsx
+++ b/Data template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\somalia macro model for CBK\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\somali economic outlook report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74D1C084-71D7-45EA-A551-54BDE651F231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF64C85A-0A1F-458D-8B4B-7C134FEB5EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Real Sector Raw" sheetId="2" r:id="rId1"/>
@@ -2861,7 +2861,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2912,6 +2912,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3502,7 +3508,9 @@
       <c r="L4" s="10">
         <v>11966</v>
       </c>
-      <c r="M4" s="10"/>
+      <c r="M4" s="13">
+        <v>12324.98</v>
+      </c>
     </row>
     <row r="5" spans="1:13" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
@@ -3541,7 +3549,9 @@
       <c r="L5" s="10">
         <v>11066</v>
       </c>
-      <c r="M5" s="6"/>
+      <c r="M5" s="13">
+        <v>11397.98</v>
+      </c>
     </row>
     <row r="6" spans="1:13" s="18" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
@@ -3680,7 +3690,9 @@
       <c r="L10" s="10">
         <v>14569</v>
       </c>
-      <c r="M10" s="6"/>
+      <c r="M10" s="6">
+        <v>15006.07</v>
+      </c>
     </row>
     <row r="11" spans="1:13" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
@@ -3719,7 +3731,9 @@
       <c r="L11" s="10">
         <v>900</v>
       </c>
-      <c r="M11" s="6"/>
+      <c r="M11" s="6">
+        <v>927</v>
+      </c>
     </row>
     <row r="12" spans="1:13" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
@@ -3758,7 +3772,9 @@
       <c r="L12" s="10">
         <v>3344</v>
       </c>
-      <c r="M12" s="6"/>
+      <c r="M12" s="6">
+        <v>3444.32</v>
+      </c>
     </row>
     <row r="13" spans="1:13" s="18" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
@@ -3822,7 +3838,9 @@
       <c r="L14" s="10">
         <v>3639</v>
       </c>
-      <c r="M14" s="6"/>
+      <c r="M14" s="6">
+        <v>3748.17</v>
+      </c>
     </row>
     <row r="15" spans="1:13" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
@@ -3861,7 +3879,9 @@
       <c r="L15" s="10">
         <v>11386</v>
       </c>
-      <c r="M15" s="6"/>
+      <c r="M15" s="6">
+        <v>11727.58</v>
+      </c>
     </row>
     <row r="16" spans="1:13" s="18" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
@@ -4164,6 +4184,7 @@
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>